<commit_message>
Update Birthday Memo data
</commit_message>
<xml_diff>
--- a/Birthdays.xlsx
+++ b/Birthdays.xlsx
@@ -3241,7 +3241,7 @@
         <v>17</v>
       </c>
       <c r="E37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="E37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">

</xml_diff>